<commit_message>
Arbitrer la sélection finale des vidéos expert et enrichir le suivi.
Consolide les positionnements intervenants, retire Joël Nguen, ajoute la matrice de cohérence, l’export XLSX dédié et les mails « vidéos attendues ».

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/suivi_positionnements.xlsx
+++ b/site/suivi_positionnements.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Suivi positionnements" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Selection finale" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Matrice coherence" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -496,7 +498,11 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -517,7 +523,11 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>E13 ; E18 ; E15</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -538,7 +548,11 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>E1 ; E20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -575,7 +589,11 @@
           <t>E22 ou E23 (prioritaire) ; E8 egalement possible</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -593,10 +611,39 @@
           <t>T3 (E4, E5) ; T6 (E10, E11) ; T7 (E12, E13, E13bis) ; T8 (E14, E15) ; T12 (E22, E23)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour Rita,
+J'espère que tu vas bien.
+Je te remercie pour ton message et te prie de m'excuser du délai de réponse.
+Après relecture du guide de travail, je souhaiterais me positionner sur les vidéos expertises suivantes :
+Vidéo expertise 5 — Objectif : Dérisquer un projet par étapes. Prématuration, maturation, jalons techniques et commerciaux, critères de décision.
+Vidéo expertise 12 — Objectif : De la prématuration à la maturation. Étapes, sélection, investissement, jalons et accompagnement.
+Vidéo expertise 14 — Objectif : La chaîne des financements de l'innovation. Prématuration, maturation, aides non dilutives, concours, Bpifrance et financement privé.
+Vidéo expertise 15 — Objectif : Comprendre la logique des investisseurs. Dilution, retour attendu, rythme de croissance, gouvernance et compatibilité avec le projet.
+Par contre, il n'y avait pas en pièce jointe du mail initial les capsules témoins concernées, en particulier T3, T7 et T8.
+Pourrais-tu s'il te plaît me les transmettre pour information ?
+Je pourrais, selon ton retour sur le positionnement retenu, te faire part de mes commentaires plus précis sur les scripts.
+Enfin, pour information, je serai absente à partir de ce soir jusqu'au 14 août inclus.
+Je reste à ta disposition pour échanger au besoin à mon retour.
+Bel été</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Demande la transmission des capsules témoins T3, T7 et T8. Souhaite commenter plus précisément les scripts après retour sur le positionnement retenu. Absente jusqu'au 14 août inclus.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>E5 ; E12 ; E14 ; E15</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>E12 ; E14</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -635,33 +682,66 @@
           <t>E3</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>E2 ; E3</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Joël Nguen</t>
+          <t>Pascal Corbel</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Organisme de rattachement à confirmer</t>
+          <t>Université Paris-Saclay</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>T10 (E18, E19) ; T11 (E20, E21)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>T9 (E16, E17) ; T10 (E18, E19) ; T11 (E20, E21)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Bonjour Rita-Noeëlle,
+Voici mon retour :
+Vidéo 16 : Oui, s'il s'agit bien d'insister sur les effets de complémentarité et la possibilité d'apprentissage et non de lister des compétences-types nécessaires ;
+Vidéo 17 : Non, un juriste me paraîtrait plus pertinent ;
+Vidéo 18 : Oui, s'il s'agit en particulier de bien distinguer technologie et proposition de valeur ; non, si l'orientation est vraiment très "communication".
+Vidéo 19 : Oui, en particulier si on peut en profiter pour déconstruire la figure de l'entrepreneur visionnaire.
+Vidéo 20 : Non, je ne pense pas être le plus qualifié pour parler de ces parcours de chercheurs-entrepreneurs.
+Vidéo 21 : Oui.
+Bien cordialement,
+Pascal Corbel,
+Professeur des Universités en sciences de gestion et du management,
+Responsable du M2 EMPI
+Université Paris-Saclay
+pascalcorbel.fr</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Souhaite un cadrage précis : E16 sur complémentarité et apprentissage ; E18 sur distinction technologie / proposition de valeur ; E19 pour déconstruire la figure de l'entrepreneur visionnaire. Estime qu'un juriste serait plus pertinent pour E17 et ne se juge pas le plus qualifié pour E20.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>E19 ; E21</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>E16 ; E19 ; E21</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Pascal Corbel</t>
+          <t>Rémi Waché</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -671,18 +751,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>T9 (E16, E17) ; T10 (E18, E19) ; T11 (E20, E21)</t>
+          <t>T12 (E22, E23)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Rémi Waché</t>
+          <t>Soizic Lefeuvre</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -692,139 +776,126 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>T12 (E22, E23)</t>
+          <t>T4 (E6, E7) ; T5 (E8, E9) ; T6 (E10, E11) ; T12 (E22, E23)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Soizic Lefeuvre</t>
+          <t>Stanislas De Lapasse</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Université Paris-Saclay</t>
+          <t>INPI</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>T4 (E6, E7) ; T5 (E8, E9) ; T6 (E10, E11) ; T12 (E22, E23)</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
+          <t>T5 (E8, E9)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Positionnement confirme sur les deux videos proposees (E8 et E9 / T5).</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>E8 ; E9 (acceptation des deux videos proposees)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>E8 ; E9</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Stanislas De Lapasse</t>
+          <t>Stephanie Oger-Roussel</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>INPI</t>
+          <t>Communication de SATT Paris-Saclay</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>T5 (E8, E9)</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Positionnement confirme sur les deux videos proposees (E8 et E9 / T5).</t>
-        </is>
-      </c>
+          <t>T3 (E4, E5) ; T6 (E10, E11) ; T7 (E12, E13, E13bis) ; T8 (E14, E15)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>E8 ; E9 (acceptation des deux videos proposees)</t>
-        </is>
-      </c>
+      <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>E8 ; E9</t>
+          <t>E4</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Stephanie Oger-Roussel</t>
+          <t>Stephanie Sano</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SATT Paris-Saclay</t>
+          <t>UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>T3 (E4, E5) ; T6 (E10, E11) ; T7 (E12, E13, E13bis) ; T8 (E14, E15)</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
+          <t>T4 (E6, E7)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 — Positionnement confirme sur les deux videos proposees (E6 et E7 / T4).</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>E6 ; E7 (acceptation des deux videos proposees)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>E6 ; E7</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Stephanie Sano</t>
+          <t>Virginia Branco</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Organisme de rattachement à confirmer</t>
+          <t>ENS Paris-Saclay</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>T4 (E6, E7)</t>
+          <t>T3 (E4, E5) ; T6 (E10, E11) ; T12 (E22, E23)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-23 — Positionnement confirme sur les deux videos proposees (E6 et E7 / T4).</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>E6 ; E7 (acceptation des deux videos proposees)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>E6 ; E7</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Virginia Branco</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>ENS Paris-Saclay</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>T3 (E4, E5) ; T6 (E10, E11) ; T12 (E22, E23)</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>2026-07-22 — Bonjour Rita,
 Je suis en congés du 24/07 au 25/08, le timing est très serré.
@@ -835,38 +906,2278 @@
 (Note saisie : « 240/07 » corrige en 24/07 dans le suivi.)</t>
         </is>
       </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Congés du 24/07 au 25/08 — timing très serré. Demande la prochaine étape.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>E10 ; E11 ; E5 ; E22 (ordre de preference)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>E10 ; E5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Yoann Montenot</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Université Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>T7 (E12, E13, E13bis)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>E13bis</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Vidéo expertise</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Objectif</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Intervenant</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Organisme</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fonction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Tech-push, market-pull, observation d'usage, rencontre, sérendipité, maturation progressive.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Bernard Yannou</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>CentraleSupélec</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Innovation / design engineering / deeptech</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 2</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Utilisateur, client, beneficiaire, usage et proposition de valeur.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Gregoire Burgé</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>AgroParisTech</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Innovation agro / transfert technologique</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 3</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Validation, hypotheses, experimentation, pivot et apprentissage.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Gregoire Burgé</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>AgroParisTech</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Innovation agro / transfert technologique</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 4</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Clarifier les niveaux de preuve.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Stephanie Oger-Roussel</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Communication de SATT Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Stratégie innovation / transfert (SATT Paris-Saclay)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 5</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Prématuration, maturation, jalons techniques et commerciaux, criteres de décision.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Virginia Branco</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ENS Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Appui recherche-innovation / transfert technologique</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 6</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Confidentialite, nouveaute, publication, congres, soutenance et DI.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Stephanie Sano</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Experte UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>E7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 7</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Premier contact, rôle du charge de valorisation et informations utiles pour examiner un résultat.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Stephanie Sano</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Experte UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>E8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 8</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Brevetabilite, secret, savoir-faire, logiciel, preuve et confidentialite.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Stanislas De Lapasse</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>INPI</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Propriété industrielle / INPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>E9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 9</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Barriere à l'entree, pouvoir de negociation, credibilite et articulation avec le modele de valorisation.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Stanislas De Lapasse</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>INPI</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Propriété industrielle / INPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 10</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Licence, création, co-développement, partenariat et criteres de choix.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Virginia Branco</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>ENS Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Appui recherche-innovation / transfert technologique</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 11</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Licence exclusive ou non, cession, contrat de collaboration, copropriete et principes de negociation.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Soizic Lefeuvre</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Université Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Partenariat et valorisation / droit contrats et PI</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>E12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 12</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Étapes, sélection, investissement, jalons et accompagnement.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Fatoumata Aonon</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>CNRS</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Valorisation recherche / accompagnement projets</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>E13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 13</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Coaching, réseau, formation, confrontation, équipe et préparation de la création.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Arielle Santé</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>IncubAlliance</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Entrepreneuriat deeptech / incubation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>E13BIS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 13 BIS</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Design spot, fablab, pole de competitivite, OTT, etc.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Yoann Montenot</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Congés du 24/07 au 25/08 — timing très serré. Demande la prochaine étape.</t>
+          <t>Université Paris-Saclay</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>E10 ; E11 ; E5 ; E22 (ordre de preference)</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
+          <t>Design d'innovation / Design Spot Paris-Saclay</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 14</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Prématuration, maturation, aides non dilutives, concours, Bpifrance et financement prive.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Fatoumata Aonon</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>CNRS</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Valorisation recherche / accompagnement projets</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>E15</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 15</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Dilution, retour attendu, rythme de croissance, gouvernance et compatibilite avec le projet.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Arielle Santé</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>IncubAlliance</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Entrepreneuriat deeptech / incubation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 16</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Complémentarité, recrutement, rôle du CEO, du CSO et du CTO, et criteres humains.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Pascal Corbel</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Université Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Management innovation / PI / entrepreneuriat</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 17</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Gouvernance, responsabilites, repartition du pouvoir, parts, pacte et prevention des conflits.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Antoine Latreille</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Université Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Droit de l'innovation / propriété industrielle</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 18</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Adapter le message selon l'utilisateur, le decideur, le partenaire ou l'investisseur.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Arielle Santé</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>IncubAlliance</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Entrepreneuriat deeptech / incubation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 19</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Feedback, entrainement, mentorat et evolution de l'identite professionnelle.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Pascal Corbel</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Université Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Management innovation / PI / entrepreneuriat</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 20</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Temps, légitimité, entourage, droit à l'apprentissage et securisation du parcours.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Bernard Yannou</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>CentraleSupélec</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Innovation / design engineering / deeptech</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 21</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Incertitude, essais, erreurs, pivot et progression plutot que reussite lineaire. Focaliser le discours sur les leviers existants pour vaincre les freins.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Pascal Corbel</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Université Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Management innovation / PI / entrepreneuriat</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 22</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Objectifs partages, complémentarité, gouvernance, engagement, création et partage de valeur.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Rémi Waché</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Université Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Développement de partenariats recherche-industrie</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 23</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Confidentialite, contrats, connaissances anterieures, résultats nouveaux, PI, publication et sortie du partenariat.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Eneli Vino</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>CNRS</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Juridique PI / contrats / valorisation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Vidéo expertise</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Objectif</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Antoine Latreille</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Arielle Santé</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Bernard Yannou</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Eneli Vino</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Fatoumata Aonon</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Gregoire Burgé</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Pascal Corbel</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Rémi Waché</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Soizic Lefeuvre</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Stanislas De Lapasse</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Stephanie Oger-Roussel</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Stephanie Sano</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Virginia Branco</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>Yoann Montenot</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tech-push, market-pull, observation d'usage, rencontre, sérendipité, maturation progressive.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Utilisateur, client, beneficiaire, usage et proposition de valeur.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Validation, hypotheses, experimentation, pivot et apprentissage.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Clarifier les niveaux de preuve.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Prématuration, maturation, jalons techniques et commerciaux, criteres de décision.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Confidentialite, nouveaute, publication, congres, soutenance et DI.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Premier contact, rôle du charge de valorisation et informations utiles pour examiner un résultat.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Brevetabilite, secret, savoir-faire, logiciel, preuve et confidentialite.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Barriere à l'entree, pouvoir de negociation, credibilite et articulation avec le modele de valorisation.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Licence, création, co-développement, partenariat et criteres de choix.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Licence exclusive ou non, cession, contrat de collaboration, copropriete et principes de negociation.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Étapes, sélection, investissement, jalons et accompagnement.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Coaching, réseau, formation, confrontation, équipe et préparation de la création.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 13 BIS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Design spot, fablab, pole de competitivite, OTT, etc.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 14</t>
+        </is>
+      </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Université Paris-Saclay</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>T7 (E12, E13, E13bis)</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
+          <t>Prématuration, maturation, aides non dilutives, concours, Bpifrance et financement prive.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 15</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Dilution, retour attendu, rythme de croissance, gouvernance et compatibilite avec le projet.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 16</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Complémentarité, recrutement, rôle du CEO, du CSO et du CTO, et criteres humains.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 17</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Gouvernance, responsabilites, repartition du pouvoir, parts, pacte et prevention des conflits.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 18</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Adapter le message selon l'utilisateur, le decideur, le partenaire ou l'investisseur.</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 19</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Feedback, entrainement, mentorat et evolution de l'identite professionnelle.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 20</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Temps, légitimité, entourage, droit à l'apprentissage et securisation du parcours.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 21</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Incertitude, essais, erreurs, pivot et progression plutot que reussite lineaire. Focaliser le discours sur les leviers existants pour vaincre les freins.</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 22</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Objectifs partages, complémentarité, gouvernance, engagement, création et partage de valeur.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo Expert 23</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Confidentialite, contrats, connaissances anterieures, résultats nouveaux, PI, publication et sortie du partenariat.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Pascal Corbel E16/E19/E21 : scripts reçus, revues annotées et mail unique.
Scripts déposés verbatim dans scripts_recus/. Revues 1 en mode annoté
(texte de l'expert intact, remarques entre parenthèses) : durée sous la
cible (E16 2 min 20, E19 2 min 50, E21 3 min 50), ancrages T9/T10/T11
disponibles et non utilisés, recouvrement E19/E21 avec deux chutes
quasi identiques soumis à l'arbitrage de l'expert, coquilles prompteur.

E21 recadré « Innover comme processus d'apprentissage » et intervenant
Pascal Corbel (Joël Nguen subsistait depuis juillet). Les freins
personnels restent portés par T13.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/suivi_positionnements.xlsx
+++ b/site/suivi_positionnements.xlsx
@@ -719,12 +719,14 @@
 Professeur des Universités en sciences de gestion et du management,
 Responsable du M2 EMPI
 Université Paris-Saclay
-pascalcorbel.fr</t>
+pascalcorbel.fr
+2026-09-03 — Trois scripts recus (E16, E19, E21) en piece jointe d'un mail a Rita-Noelle Faucon : « Vous trouverez en piece jointe une proposition de script pour les 3 sequences video. N'hesitez pas a faires remarques et a me dire si cela ne correspond pas tout a fait aux attentes. » Remercie pour les informations pratiques. Chaque script est precede d'une ligne de cadrage rappelant la video temoin associee et l'angle retenu (complementarite et apprentissage pour E16 ; deconstruction de la figure de l'entrepreneur visionnaire pour E19 ; essais, erreurs, pivot et leviers pour E21).</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Souhaite un cadrage précis : E16 sur complémentarité et apprentissage ; E18 sur distinction technologie / proposition de valeur ; E19 pour déconstruire la figure de l'entrepreneur visionnaire. Estime qu'un juriste serait plus pertinent pour E17 et ne se juge pas le plus qualifié pour E20.</t>
+          <t>Souhaite un cadrage précis : E16 sur complémentarité et apprentissage ; E18 sur distinction technologie / proposition de valeur ; E19 pour déconstruire la figure de l'entrepreneur visionnaire. Estime qu'un juriste serait plus pertinent pour E17 et ne se juge pas le plus qualifié pour E20.
+2026-09-03 — Demande des remarques et une confirmation d'adequation aux attentes. Points de retour de notre cote : duree en dessous de la cible (E16 2 min 20, E19 2 min 50, E21 3 min 50 pour 5 min +/- 2) ; absence d'ancrage sur les temoignages montes T9/T10/T11 ; recouvrement entre la conclusion de E19 et l'ensemble de E21, avec deux chutes quasi identiques ; presentation de l'intervenant manquante ; coquilles a corriger avant prompteur. Revues annotees E16/E19/E21 et mail unique prets a envoyer.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1693,7 +1695,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Temps, légitimité, entourage, doute ; incertitude, essais, pivot ; première action reversible.</t>
+          <t>Incertitude, essais, erreurs, pivot et progression plutot que reussite lineaire ; leviers existants pour depasser les freins.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -3032,7 +3034,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Temps, légitimité, entourage, doute ; incertitude, essais, pivot ; première action reversible.</t>
+          <t>Incertitude, essais, erreurs, pivot et progression plutot que reussite lineaire ; leviers existants pour depasser les freins.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">

</xml_diff>

<commit_message>
Mail Pascal Corbel : apercus des montages temoins, usage de l'IA assume, choix du texte laisse a l'expert
</commit_message>
<xml_diff>
--- a/site/suivi_positionnements.xlsx
+++ b/site/suivi_positionnements.xlsx
@@ -1439,7 +1439,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Design spot, fablab, pole de competitivite, OTT, etc.</t>
+          <t>Design spot, fablab, pole de competitivite, OTT, etc. — pour les start-up de nos chercheurs, pas des start-up generiques.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Design spot, fablab, pole de competitivite, OTT, etc.</t>
+          <t>Design spot, fablab, pole de competitivite, OTT, etc. — pour les start-up de nos chercheurs, pas des start-up generiques.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">

</xml_diff>